<commit_message>
defect-hub: update tracking for Smartshift Defect.xlsx (1/2 ticketed)
</commit_message>
<xml_diff>
--- a/tracking/2026-10-30/a95933f5-8c3a-43de-a63d-239328c01f77_Smartshift Defect.xlsx
+++ b/tracking/2026-10-30/a95933f5-8c3a-43de-a63d-239328c01f77_Smartshift Defect.xlsx
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="66">
   <si>
     <t>Customer</t>
   </si>
@@ -245,34 +245,46 @@
     <t>mkarthik@smartshift.com</t>
   </si>
   <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>attachments/samples/st22_cast_dump.png|attachments/samples/analysis_cast_error.docx</t>
+  </si>
+  <si>
+    <t>JAIT-15</t>
+  </si>
+  <si>
+    <t>PROCESSED</t>
+  </si>
+  <si>
+    <t>2026-10-30T07:08:06.817Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Orica</t>
+  </si>
+  <si>
+    <t>Duplicate records showing in excel</t>
+  </si>
+  <si>
+    <t>Shows Duplicate entries on multiple projects</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>attachments/samples/st22_cast_dump.png|attachments/samples/analysis_cast_error.docx</t>
-  </si>
-  <si>
-    <t/>
+    <t>attachments/samples/cds_duplicate_rows.png|attachments/samples/cds_row_counts.xlsx</t>
   </si>
   <si>
     <t>PENDING</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Orica</t>
-  </si>
-  <si>
-    <t>Duplicate records showing in excel</t>
-  </si>
-  <si>
-    <t>Shows Duplicate entries on multiple projects</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>attachments/samples/cds_duplicate_rows.png|attachments/samples/cds_row_counts.xlsx</t>
   </si>
   <si>
     <t>File / link</t>
@@ -879,21 +891,21 @@
         <v>32</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
@@ -905,10 +917,10 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G3" t="s">
         <v>25</v>
@@ -917,7 +929,7 @@
         <v>26</v>
       </c>
       <c r="I3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J3" t="s">
         <v>28</v>
@@ -926,28 +938,28 @@
         <v>28</v>
       </c>
       <c r="L3" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="M3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="N3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O3" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
       <c r="R3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -979,16 +991,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -999,16 +1011,16 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1019,56 +1031,56 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1095,35 +1107,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>